<commit_message>
Latest Hire code After Regresion PK17
</commit_message>
<xml_diff>
--- a/Data/27/Workday_NewHire_Belgium_Regression_PK17.xlsx
+++ b/Data/27/Workday_NewHire_Belgium_Regression_PK17.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="131">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -214,7 +214,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10699415</t>
+    <t>10699517</t>
   </si>
   <si>
     <t>Passed</t>
@@ -229,10 +229,10 @@
     <t>Mr</t>
   </si>
   <si>
-    <t>Quinton</t>
-  </si>
-  <si>
-    <t>Bechtelar</t>
+    <t>Marlin</t>
+  </si>
+  <si>
+    <t>Hayes</t>
   </si>
   <si>
     <t>Landline</t>
@@ -364,392 +364,7 @@
     <t>Test2</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Berenice Casper' Employee:{10699417}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for getByRole('tablist').getByText('Pay Group')[22m
-[2m  -   locator resolved to &lt;div class="gwt-Label WO4-" data-automation-id="tabLa…&gt;Pay Group&lt;/div&gt;[22m
-[2m  - attempting click action[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #1[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #2[22m
-[2m  -   waiting 20ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #3[22m
-[2m  -   waiting 100ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #4[22m
-[2m  -   waiting 100ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #5[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #6[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #7[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #8[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #9[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #10[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #11[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #12[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #13[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #14[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #15[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #16[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #17[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #18[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #19[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #20[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #21[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #22[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #23[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #24[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #25[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #26[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #27[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #28[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #29[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #30[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #31[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #32[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #33[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #34[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #35[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #36[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #37[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #38[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #39[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #40[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #41[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #42[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #43[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #44[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #45[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #46[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #47[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #48[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #49[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #50[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #51[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #52[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #53[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is visible, enabled and stable[22m
-[2m  -   scrolling into view if needed[22m
-[2m  -   done scrolling[22m
-[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
-[2m  - retrying click action, attempt #54[22m
-[2m  -   waiting 500ms[22m
-</t>
-  </si>
-  <si>
-    <t>Failed</t>
+    <t>10699516</t>
   </si>
   <si>
     <t>751 Store Management (Rykec Puvyjo (10528834))</t>
@@ -758,13 +373,13 @@
     <t>Mme</t>
   </si>
   <si>
-    <t>Berenice</t>
-  </si>
-  <si>
-    <t>Casper</t>
-  </si>
-  <si>
-    <t>Auto 74973280</t>
+    <t>Elisa</t>
+  </si>
+  <si>
+    <t>Reilly</t>
+  </si>
+  <si>
+    <t>Auto 17476992</t>
   </si>
   <si>
     <t>Fixed Term (Fixed Term)</t>
@@ -878,7 +493,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1641,7 +1256,7 @@
       </c>
       <c r="L2" s="19">
         <f t="shared" ref="L2" si="0">TODAY()-31</f>
-        <v>45774</v>
+        <v>45779</v>
       </c>
       <c r="M2" s="14" t="s">
         <v>69</v>
@@ -1675,7 +1290,7 @@
       </c>
       <c r="W2" s="23">
         <f t="shared" ref="W2" si="1">L2</f>
-        <v>45774</v>
+        <v>45779</v>
       </c>
       <c r="X2" s="18" t="s">
         <v>80</v>
@@ -1727,7 +1342,7 @@
       </c>
       <c r="AN2" s="1">
         <f t="array" ref="AN2:AN3">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>28393076920</v>
+        <v>81529132415</v>
       </c>
       <c r="AO2" s="14" t="s">
         <v>93</v>
@@ -1819,26 +1434,26 @@
       <c r="A3" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="1" t="s">
         <v>116</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>117</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>118</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>69</v>
       </c>
       <c r="F3" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G3" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="H3" s="17" t="s">
         <v>120</v>
-      </c>
-      <c r="H3" s="17" t="s">
-        <v>121</v>
       </c>
       <c r="I3" s="18">
         <v>25041111</v>
@@ -1851,7 +1466,7 @@
       </c>
       <c r="L3" s="19">
         <f t="shared" ref="L3" si="2">TODAY()-31</f>
-        <v>45774</v>
+        <v>45779</v>
       </c>
       <c r="M3" s="14" t="s">
         <v>69</v>
@@ -1885,19 +1500,19 @@
       </c>
       <c r="W3" s="23">
         <f t="shared" ref="W3" si="3">L3</f>
-        <v>45774</v>
+        <v>45779</v>
       </c>
       <c r="X3" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y3" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="Z3" t="s">
         <v>122</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" s="25" t="s">
         <v>123</v>
-      </c>
-      <c r="AA3" s="25" t="s">
-        <v>124</v>
       </c>
       <c r="AB3" t="s">
         <v>84</v>
@@ -1912,20 +1527,20 @@
         <v>35</v>
       </c>
       <c r="AF3" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG3" t="s">
         <v>87</v>
       </c>
       <c r="AH3" s="19">
         <f>TODAY()+365</f>
-        <v>46170</v>
+        <v>46175</v>
       </c>
       <c r="AI3" s="18" t="s">
         <v>89</v>
       </c>
       <c r="AJ3" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK3" s="1">
         <v>251</v>
@@ -1937,23 +1552,23 @@
         <v>92</v>
       </c>
       <c r="AN3" s="1">
-        <v>12838024449</v>
+        <v>64811399547</v>
       </c>
       <c r="AO3" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP3" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AQ3" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR3" s="19">
         <f t="shared" ref="AR3" si="4">AH3</f>
-        <v>46170</v>
+        <v>46175</v>
       </c>
       <c r="AS3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AT3" s="29">
         <v>35591</v>
@@ -1980,10 +1595,10 @@
         <v>69</v>
       </c>
       <c r="BB3" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="BC3" t="s">
         <v>128</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>129</v>
       </c>
       <c r="BD3" s="14" t="s">
         <v>102</v>
@@ -2004,10 +1619,10 @@
         <v>107</v>
       </c>
       <c r="BJ3" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK3" s="30" t="s">
         <v>130</v>
-      </c>
-      <c r="BK3" s="30" t="s">
-        <v>131</v>
       </c>
       <c r="BL3" s="30" t="s">
         <v>110</v>

</xml_diff>